<commit_message>
Add GEO accession + publication DOI columns to data summary workbook
Verified GEO/BioProject and DOIs against NCBI and source papers; fixed nagano cell type (Th1) and droplethic (human cell-line mixing)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/summary/benchmark_data_summary.xlsx
+++ b/summary/benchmark_data_summary.xlsx
@@ -493,20 +493,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,40 +536,50 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Publication DOI</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Genome</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Cell type / tissue</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Modalities</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Cells listed</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Cells used in benchmark</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>SRA / GEO accessions</t>
-        </is>
-      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>GEO accession</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>SRA accessions</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
           <t>Pipeline / aligner</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Role &amp; notes</t>
         </is>
@@ -586,45 +598,55 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>This study</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+          <t>This study (unpublished)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>hg38</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>GM12878 (lymphoblastoid cell line)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>CpG meth (HCG) + GpC accessibility (GCH) + Hi-C</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>188</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>187 (QC-pass)</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>-  (not yet deposited)</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>In-house (scNH_GM_4plex_*); bhmem output external at b1198 gm_sc_new</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>TrimGalore -&gt; bhmem (bisulfitehic BWA-MEM) -&gt; markdup/calmd; YAP bowtie2 arm as local comparison</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>The published method being benchmarked. Three modalities. bhmem is the method aligner (external); local YAP/bowtie2 arm feeds mapping/Hi-C QC.</t>
         </is>
@@ -643,45 +665,55 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Nagano et al. 2013</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+          <t>Nagano et al. 2013, Nature</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>10.1038/nature12593</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>mm10</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Mouse ESC (single cells)</t>
-        </is>
-      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
+          <t>Mouse Th1 cells (single cells)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>Hi-C only (no methylation)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>GSE48262</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>SRR921526-SRR921540</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>fastp -&gt; bwa-mem2 -SP5M -&gt; samtools markdup -&gt; pairtools</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>Early pure scHi-C reference. High trans_ratio (~0.17) is a real quality signature of this early assay.</t>
         </is>
@@ -700,45 +732,55 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Chang et al. 2025</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
+          <t>Chang et al. 2025, Nat Biotechnol</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>10.1038/s41587-024-02447-1</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>hg38</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Cell line (barcoded droplets)</t>
-        </is>
-      </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
+          <t>Human cell-line mixing (barcoded droplets)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
           <t>Hi-C only</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>~688k barcodes</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>3,668 valid barcodes</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>GSE253407 (PRJNA1065475)</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>SRR27586278, SRR27586279</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>Rupture: TrimGalore -&gt; bowtie1 barcode -&gt; bwa mem -SP5M -&gt; CB-tag -&gt; pairtools</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>High-throughput droplet Hi-C. CAVEAT: pairtools dedup not run -&gt; values are currently pre-dedup (kept as-is by decision 2026-06-30).</t>
         </is>
@@ -757,45 +799,55 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Pott 2017</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+          <t>Pott 2017, eLife</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>10.7554/eLife.23203</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>hg38</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>GM12878 + K562 (cell lines)</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>CpG meth (HCG) + GpC accessibility (GCH); no Hi-C</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>34 runs (after control removal)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>23 cells (12 GM12878 + 11 merged K562)</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>GSE83882</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>SRR3729642-SRR3729653 (GM12878); SRR3729661-SRR3729682 (K562); SRR3729654-3729660 = excluded spike-in controls</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>TrimGalore -&gt; Bismark SE per-mate (--non_directional) -&gt; markdup -&gt; coverage2cytosine --nome-seq</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>NOMe method (CpG + GCH accessibility). K562 has 2 runs/cell merged into 11 cells; controls excluded.</t>
         </is>
@@ -814,45 +866,55 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Luo 2018</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
+          <t>Luo et al. 2018, Nat Commun</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>10.1038/s41467-018-06355-2</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>hg38 + mm10</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Mixed species single cells</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>CpG methylation only (not NOMe, no GCH); no Hi-C</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>249 (153 hg38 + 96 mm10)</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>mm10 subset = 96</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>GSE112471</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>SRR6911624 ... (250-line acc_list)</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="L8" s="8" t="inlineStr">
         <is>
           <t>cutadapt -&gt; Bismark SE per-mate -&gt; dedup -&gt; methyl-extractor; parallel YAP mc arm</t>
         </is>
       </c>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>CpG-only methylome. mm10 subset used for the benchmark figures.</t>
         </is>
@@ -871,45 +933,55 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Liu 2023</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+          <t>Liu et al. 2023, Nature</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>10.1038/s41586-023-06805-y</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>mm10</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Mouse single cells</t>
-        </is>
-      </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Mouse brain (single nuclei)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>CpG methylation + Hi-C (m3C chimeric split-read contacts)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>1,379 in SRA pool (100 aligned)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>GSE213259 (PRJNA880294)</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>SRR21549289 ... (1379-line acc_list)</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>cutadapt -&gt; YAP bismark+bowtie2 m3C (alignment/) AND bhmem (04.bhmem_bam/)</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>Combined methylome + Hi-C. Final figures: align+contacts from YAP, conversion+HCG loci from bhmem. Contacts are chimeric multi-way (method-inherent difference).</t>
         </is>
@@ -928,45 +1000,55 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Smallwood 2014</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+          <t>Smallwood et al. 2014, Nat Methods</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>10.1038/nmeth.3035</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>mm10</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Mouse ESC (single cells)</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>CpG methylation only (WGBS); no Hi-C, no GCH</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>51</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>51</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>GSE56879</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>SRR1248444 ... (51-line acc_list)</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>TrimGalore -&gt; Bismark (hg38 contamination depletion -&gt; mm10 SE) -&gt; markdup -&gt; cov + BisSNP</t>
         </is>
       </c>
-      <c r="K10" s="8" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Whole-genome bisulfite single-cell reference (no accessibility, no Hi-C).</t>
         </is>
@@ -985,45 +1067,55 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Luo 2022</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+          <t>Luo et al. 2022, Cell Genomics</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>10.1016/j.xgen.2022.100107</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>hg38</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Human frontal cortex, donor UMB5580 (batch 190321)</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>CpG meth (HCG) + GpC accessibility (GCH) + RNA (transcriptome)</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>99</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>GSE140493 (SRR* per cells_brain.tsv)</t>
-        </is>
-      </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
+          <t>GSE140493</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>SRR* per cells_brain.tsv (subset of GSE140493)</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
           <t>YAP mct --nome (bismark methylome + STAR transcriptome + allcools)</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Multi-omic NOMe brain data. NB: autosomal non-CpG is elevated by real brain neuronal mCH, not conversion failure. Median HCG 81.2% / GCH 15.1%.</t>
         </is>
@@ -1042,45 +1134,55 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Li et al. 2019</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+          <t>Li et al. 2019, Nat Methods</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>10.1038/s41592-019-0502-z</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>mm10</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Single cells</t>
-        </is>
-      </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
+          <t>Mouse ESC (single cells)</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
           <t>CpG methylation + Hi-C</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Excluded from current figures</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>GSE119171</t>
+        </is>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>SRR7770822 ... (59-line acc_list)</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="L12" s="10" t="inlineStr">
         <is>
           <t>YAP (m3C)</t>
         </is>
       </c>
-      <c r="K12" s="10" t="inlineStr">
+      <c r="M12" s="10" t="inlineStr">
         <is>
           <t>Excluded from the current benchmark figures per user decision.</t>
         </is>
@@ -1099,47 +1201,57 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Li et al. 2019 (newer batch)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
+          <t>Methyl-HiC (in-house batch)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>10.1038/s41592-019-0502-z (method)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>mm10</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Single cells</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>CpG methylation + Hi-C</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>96</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>Excluded from current figures</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>In-house (not deposited; Novogene CKDL IDs)</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>In-house sample IDs (sc_*_CKDL*, 96-line acc_list)</t>
         </is>
       </c>
-      <c r="J13" s="10" t="inlineStr">
+      <c r="L13" s="10" t="inlineStr">
         <is>
           <t>Snakemake per-Group alignment</t>
         </is>
       </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>Newer Methyl-HiC batch; also excluded from current benchmark figures per user decision.</t>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>Newer Methyl-HiC batch; also excluded from the current benchmark figures per user decision.</t>
         </is>
       </c>
     </row>

</xml_diff>